<commit_message>
Aggiornamento app Jamsetgemini: nuove funzionalità database e UI
</commit_message>
<xml_diff>
--- a/Assets/ElencoVolumiInVecchioDB.xlsx
+++ b/Assets/ElencoVolumiInVecchioDB.xlsx
@@ -5,14 +5,14 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DBSpartiti2\jamset\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\jamsetgemini\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="12960" windowHeight="5790"/>
   </bookViews>
   <sheets>
-    <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
+    <sheet name="Elenco" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="221">
   <si>
     <t>Aebersold</t>
   </si>
@@ -681,6 +681,12 @@
   </si>
   <si>
     <t>totali</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>NumBrani</t>
   </si>
 </sst>
 </file>
@@ -1010,7 +1016,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F209"/>
+  <dimension ref="A1:F210"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" customWidth="1"/>
@@ -1018,17 +1024,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
       <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1">
-        <v>12</v>
-      </c>
-      <c r="E1">
-        <v>1</v>
+        <v>219</v>
+      </c>
+      <c r="C1" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1036,13 +1036,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1050,13 +1050,13 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3">
         <v>37</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1064,13 +1064,13 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4">
-        <v>89</v>
+        <v>37</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1078,13 +1078,13 @@
         <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1092,13 +1092,13 @@
         <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="E6">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1106,13 +1106,13 @@
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="E7">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -1120,13 +1120,13 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E8">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -1134,13 +1134,13 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9">
-        <v>53</v>
+        <v>14</v>
       </c>
       <c r="E9">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -1148,13 +1148,13 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="E10">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1162,13 +1162,13 @@
         <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E11">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -1176,13 +1176,13 @@
         <v>0</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12">
         <v>13</v>
       </c>
       <c r="E12">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -1190,13 +1190,13 @@
         <v>0</v>
       </c>
       <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13">
         <v>13</v>
       </c>
-      <c r="C13">
-        <v>37</v>
-      </c>
       <c r="E13">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -1204,13 +1204,13 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="E14">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1218,13 +1218,13 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1232,13 +1232,13 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C16">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E16">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1246,13 +1246,13 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E17">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1260,13 +1260,13 @@
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="E18">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1274,13 +1274,13 @@
         <v>0</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C19">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="E19">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1288,13 +1288,13 @@
         <v>0</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C20">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E20">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1302,13 +1302,13 @@
         <v>0</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C21">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E21">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1316,13 +1316,13 @@
         <v>0</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C22">
+        <v>29</v>
+      </c>
+      <c r="E22">
         <v>21</v>
-      </c>
-      <c r="E22">
-        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1330,13 +1330,13 @@
         <v>0</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C23">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E23">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1344,13 +1344,13 @@
         <v>0</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C24">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E24">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1358,13 +1358,13 @@
         <v>0</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C25">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E25">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1372,13 +1372,13 @@
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1386,13 +1386,13 @@
         <v>0</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C27">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="E27">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1400,13 +1400,13 @@
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C28">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="E28">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1414,13 +1414,13 @@
         <v>0</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C29">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E29">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1428,13 +1428,13 @@
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C30">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E30">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1442,13 +1442,13 @@
         <v>0</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C31">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="E31">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1456,13 +1456,13 @@
         <v>0</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C32">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="E32">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1470,13 +1470,13 @@
         <v>0</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C33">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E33">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1484,13 +1484,13 @@
         <v>0</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C34">
         <v>11</v>
       </c>
       <c r="E34">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1498,13 +1498,13 @@
         <v>0</v>
       </c>
       <c r="B35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C35">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E35">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1512,13 +1512,13 @@
         <v>0</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C36">
         <v>13</v>
       </c>
       <c r="E36">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1526,13 +1526,13 @@
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C37">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="E37">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1540,13 +1540,13 @@
         <v>0</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C38">
-        <v>13</v>
+        <v>49</v>
       </c>
       <c r="E38">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1554,13 +1554,13 @@
         <v>0</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C39">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E39">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1568,13 +1568,13 @@
         <v>0</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C40">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E40">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1582,13 +1582,13 @@
         <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C41">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E41">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1596,13 +1596,13 @@
         <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C42">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E42">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1610,13 +1610,13 @@
         <v>0</v>
       </c>
       <c r="B43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C43">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E43">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1624,13 +1624,13 @@
         <v>0</v>
       </c>
       <c r="B44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C44">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="E44">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1638,13 +1638,13 @@
         <v>0</v>
       </c>
       <c r="B45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C45">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="E45">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1652,13 +1652,13 @@
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C46">
         <v>13</v>
       </c>
       <c r="E46">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -1666,13 +1666,13 @@
         <v>0</v>
       </c>
       <c r="B47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C47">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E47">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1680,13 +1680,13 @@
         <v>0</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C48">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E48">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -1694,13 +1694,13 @@
         <v>0</v>
       </c>
       <c r="B49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C49">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="E49">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -1708,13 +1708,13 @@
         <v>0</v>
       </c>
       <c r="B50" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C50">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E50">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -1722,13 +1722,13 @@
         <v>0</v>
       </c>
       <c r="B51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C51">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E51">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -1736,13 +1736,13 @@
         <v>0</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C52">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E52">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -1750,13 +1750,13 @@
         <v>0</v>
       </c>
       <c r="B53" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C53">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E53">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -1764,13 +1764,13 @@
         <v>0</v>
       </c>
       <c r="B54" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C54">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E54">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1778,13 +1778,13 @@
         <v>0</v>
       </c>
       <c r="B55" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C55">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E55">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -1792,13 +1792,13 @@
         <v>0</v>
       </c>
       <c r="B56" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C56">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E56">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -1806,13 +1806,13 @@
         <v>0</v>
       </c>
       <c r="B57" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C57">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E57">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -1820,13 +1820,13 @@
         <v>0</v>
       </c>
       <c r="B58" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C58">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="E58">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
@@ -1834,13 +1834,13 @@
         <v>0</v>
       </c>
       <c r="B59" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C59">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E59">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -1848,13 +1848,13 @@
         <v>0</v>
       </c>
       <c r="B60" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C60">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E60">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -1862,13 +1862,13 @@
         <v>0</v>
       </c>
       <c r="B61" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C61">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E61">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -1876,13 +1876,13 @@
         <v>0</v>
       </c>
       <c r="B62" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C62">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E62">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -1890,13 +1890,13 @@
         <v>0</v>
       </c>
       <c r="B63" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C63">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E63">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -1904,13 +1904,13 @@
         <v>0</v>
       </c>
       <c r="B64" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C64">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E64">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
@@ -1918,13 +1918,13 @@
         <v>0</v>
       </c>
       <c r="B65" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C65">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E65">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -1932,13 +1932,13 @@
         <v>0</v>
       </c>
       <c r="B66" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C66">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="E66">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -1946,13 +1946,13 @@
         <v>0</v>
       </c>
       <c r="B67" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C67">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E67">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
@@ -1960,13 +1960,13 @@
         <v>0</v>
       </c>
       <c r="B68" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C68">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E68">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -1974,13 +1974,13 @@
         <v>0</v>
       </c>
       <c r="B69" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C69">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E69">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -1988,13 +1988,13 @@
         <v>0</v>
       </c>
       <c r="B70" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C70">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E70">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -2002,13 +2002,13 @@
         <v>0</v>
       </c>
       <c r="B71" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C71">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E71">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -2016,13 +2016,13 @@
         <v>0</v>
       </c>
       <c r="B72" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C72">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E72">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -2030,13 +2030,13 @@
         <v>0</v>
       </c>
       <c r="B73" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C73">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E73">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -2044,13 +2044,13 @@
         <v>0</v>
       </c>
       <c r="B74" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C74">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E74">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -2058,13 +2058,13 @@
         <v>0</v>
       </c>
       <c r="B75" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C75">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E75">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -2072,13 +2072,13 @@
         <v>0</v>
       </c>
       <c r="B76" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C76">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E76">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -2086,13 +2086,13 @@
         <v>0</v>
       </c>
       <c r="B77" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C77">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="E77">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
@@ -2100,13 +2100,13 @@
         <v>0</v>
       </c>
       <c r="B78" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C78">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="E78">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -2114,13 +2114,13 @@
         <v>0</v>
       </c>
       <c r="B79" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C79">
         <v>55</v>
       </c>
       <c r="E79">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -2128,13 +2128,13 @@
         <v>0</v>
       </c>
       <c r="B80" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C80">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="E80">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="B81" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C81">
         <v>10</v>
       </c>
       <c r="E81">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -2156,13 +2156,13 @@
         <v>0</v>
       </c>
       <c r="B82" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C82">
         <v>10</v>
       </c>
       <c r="E82">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -2170,13 +2170,13 @@
         <v>0</v>
       </c>
       <c r="B83" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C83">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="E83">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -2184,13 +2184,13 @@
         <v>0</v>
       </c>
       <c r="B84" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C84">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="E84">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -2198,13 +2198,13 @@
         <v>0</v>
       </c>
       <c r="B85" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C85">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="E85">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -2212,13 +2212,13 @@
         <v>0</v>
       </c>
       <c r="B86" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C86">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="E86">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -2226,13 +2226,13 @@
         <v>0</v>
       </c>
       <c r="B87" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C87">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E87">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -2240,13 +2240,13 @@
         <v>0</v>
       </c>
       <c r="B88" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C88">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="E88">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
@@ -2254,13 +2254,13 @@
         <v>0</v>
       </c>
       <c r="B89" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C89">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E89">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -2268,13 +2268,13 @@
         <v>0</v>
       </c>
       <c r="B90" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C90">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="E90">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -2282,13 +2282,13 @@
         <v>0</v>
       </c>
       <c r="B91" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C91">
         <v>10</v>
       </c>
       <c r="E91">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -2296,13 +2296,13 @@
         <v>0</v>
       </c>
       <c r="B92" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C92">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E92">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -2310,13 +2310,13 @@
         <v>0</v>
       </c>
       <c r="B93" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C93">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E93">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -2324,13 +2324,13 @@
         <v>0</v>
       </c>
       <c r="B94" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C94">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E94">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
@@ -2338,13 +2338,13 @@
         <v>0</v>
       </c>
       <c r="B95" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C95">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E95">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -2352,13 +2352,13 @@
         <v>0</v>
       </c>
       <c r="B96" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C96">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E96">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -2366,13 +2366,13 @@
         <v>0</v>
       </c>
       <c r="B97" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C97">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E97">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -2380,13 +2380,13 @@
         <v>0</v>
       </c>
       <c r="B98" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C98">
         <v>13</v>
       </c>
       <c r="E98">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -2394,13 +2394,13 @@
         <v>0</v>
       </c>
       <c r="B99" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C99">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="E99">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -2408,13 +2408,13 @@
         <v>0</v>
       </c>
       <c r="B100" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C100">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E100">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -2422,13 +2422,13 @@
         <v>0</v>
       </c>
       <c r="B101" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C101">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E101">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -2436,13 +2436,13 @@
         <v>0</v>
       </c>
       <c r="B102" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C102">
         <v>40</v>
       </c>
       <c r="E102">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -2450,13 +2450,13 @@
         <v>0</v>
       </c>
       <c r="B103" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C103">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E103">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -2464,13 +2464,13 @@
         <v>0</v>
       </c>
       <c r="B104" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C104">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="E104">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -2478,46 +2478,46 @@
         <v>0</v>
       </c>
       <c r="B105" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C105">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="E105">
-        <v>105</v>
-      </c>
-      <c r="F105" s="1">
-        <f>SUM(C1:C105)</f>
-        <v>2134</v>
+        <v>104</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="B106" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C106">
-        <v>1687</v>
+        <v>9</v>
+      </c>
+      <c r="E106">
+        <v>105</v>
       </c>
       <c r="F106" s="1">
-        <f>SUM(C106)</f>
-        <v>1687</v>
+        <f>SUM(C2:C106)</f>
+        <v>2134</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C107">
-        <v>201</v>
-      </c>
-      <c r="E107">
-        <v>1</v>
+        <v>1687</v>
+      </c>
+      <c r="F107" s="1">
+        <f>SUM(C107)</f>
+        <v>1687</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -2525,13 +2525,13 @@
         <v>108</v>
       </c>
       <c r="B108" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C108">
-        <v>13</v>
+        <v>201</v>
       </c>
       <c r="E108">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -2539,13 +2539,13 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C109">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E109">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -2553,13 +2553,13 @@
         <v>108</v>
       </c>
       <c r="B110" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C110">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E110">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -2567,13 +2567,13 @@
         <v>108</v>
       </c>
       <c r="B111" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C111">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E111">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -2581,13 +2581,13 @@
         <v>108</v>
       </c>
       <c r="B112" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C112">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E112">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
@@ -2595,13 +2595,13 @@
         <v>108</v>
       </c>
       <c r="B113" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C113">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="E113">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
@@ -2609,13 +2609,13 @@
         <v>108</v>
       </c>
       <c r="B114" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C114">
         <v>12</v>
       </c>
       <c r="E114">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
@@ -2623,13 +2623,13 @@
         <v>108</v>
       </c>
       <c r="B115" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C115">
         <v>12</v>
       </c>
       <c r="E115">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
@@ -2637,13 +2637,13 @@
         <v>108</v>
       </c>
       <c r="B116" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C116">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="E116">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
@@ -2651,13 +2651,13 @@
         <v>108</v>
       </c>
       <c r="B117" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C117">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="E117">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
@@ -2665,13 +2665,13 @@
         <v>108</v>
       </c>
       <c r="B118" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C118">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="E118">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
@@ -2679,13 +2679,13 @@
         <v>108</v>
       </c>
       <c r="B119" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C119">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E119">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
@@ -2693,13 +2693,13 @@
         <v>108</v>
       </c>
       <c r="B120" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C120">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="E120">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
@@ -2707,13 +2707,13 @@
         <v>108</v>
       </c>
       <c r="B121" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C121">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E121">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
@@ -2721,13 +2721,13 @@
         <v>108</v>
       </c>
       <c r="B122" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C122">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E122">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
@@ -2735,13 +2735,13 @@
         <v>108</v>
       </c>
       <c r="B123" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C123">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="E123">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
@@ -2749,13 +2749,13 @@
         <v>108</v>
       </c>
       <c r="B124" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C124">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E124">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
@@ -2763,13 +2763,13 @@
         <v>108</v>
       </c>
       <c r="B125" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C125">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="E125">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
@@ -2777,13 +2777,13 @@
         <v>108</v>
       </c>
       <c r="B126" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C126">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E126">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
@@ -2791,13 +2791,13 @@
         <v>108</v>
       </c>
       <c r="B127" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C127">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="E127">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
@@ -2805,13 +2805,13 @@
         <v>108</v>
       </c>
       <c r="B128" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C128">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E128">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
@@ -2819,27 +2819,27 @@
         <v>108</v>
       </c>
       <c r="B129" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C129">
-        <v>107</v>
+        <v>15</v>
       </c>
       <c r="E129">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="B130" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C130">
-        <v>41</v>
+        <v>107</v>
       </c>
       <c r="E130">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
@@ -2847,13 +2847,13 @@
         <v>132</v>
       </c>
       <c r="B131" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C131">
         <v>41</v>
       </c>
       <c r="E131">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
@@ -2861,13 +2861,13 @@
         <v>132</v>
       </c>
       <c r="B132" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C132">
         <v>41</v>
       </c>
       <c r="E132">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
@@ -2875,13 +2875,13 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C133">
         <v>41</v>
       </c>
       <c r="E133">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
@@ -2889,13 +2889,13 @@
         <v>132</v>
       </c>
       <c r="B134" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C134">
         <v>41</v>
       </c>
       <c r="E134">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
@@ -2903,13 +2903,13 @@
         <v>132</v>
       </c>
       <c r="B135" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C135">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="E135">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
@@ -2917,13 +2917,13 @@
         <v>132</v>
       </c>
       <c r="B136" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C136">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="E136">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
@@ -2931,13 +2931,13 @@
         <v>132</v>
       </c>
       <c r="B137" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C137">
         <v>41</v>
       </c>
       <c r="E137">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
@@ -2945,13 +2945,13 @@
         <v>132</v>
       </c>
       <c r="B138" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C138">
         <v>41</v>
       </c>
       <c r="E138">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
@@ -2959,13 +2959,13 @@
         <v>132</v>
       </c>
       <c r="B139" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C139">
         <v>41</v>
       </c>
       <c r="E139">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
@@ -2973,13 +2973,13 @@
         <v>132</v>
       </c>
       <c r="B140" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C140">
         <v>41</v>
       </c>
       <c r="E140">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
@@ -2987,13 +2987,13 @@
         <v>132</v>
       </c>
       <c r="B141" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C141">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E141">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
@@ -3001,13 +3001,13 @@
         <v>132</v>
       </c>
       <c r="B142" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C142">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E142">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
@@ -3015,13 +3015,13 @@
         <v>132</v>
       </c>
       <c r="B143" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C143">
         <v>41</v>
       </c>
       <c r="E143">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
@@ -3029,13 +3029,13 @@
         <v>132</v>
       </c>
       <c r="B144" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C144">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="E144">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
@@ -3043,13 +3043,13 @@
         <v>132</v>
       </c>
       <c r="B145" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C145">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E145">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
@@ -3057,13 +3057,13 @@
         <v>132</v>
       </c>
       <c r="B146" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C146">
         <v>41</v>
       </c>
       <c r="E146">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
@@ -3071,13 +3071,13 @@
         <v>132</v>
       </c>
       <c r="B147" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C147">
         <v>41</v>
       </c>
       <c r="E147">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
@@ -3085,13 +3085,13 @@
         <v>132</v>
       </c>
       <c r="B148" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C148">
         <v>41</v>
       </c>
       <c r="E148">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
@@ -3099,13 +3099,13 @@
         <v>132</v>
       </c>
       <c r="B149" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C149">
         <v>41</v>
       </c>
       <c r="E149">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
@@ -3113,13 +3113,13 @@
         <v>132</v>
       </c>
       <c r="B150" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C150">
         <v>41</v>
       </c>
       <c r="E150">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
@@ -3127,13 +3127,13 @@
         <v>132</v>
       </c>
       <c r="B151" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C151">
         <v>41</v>
       </c>
       <c r="E151">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
@@ -3141,13 +3141,13 @@
         <v>132</v>
       </c>
       <c r="B152" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C152">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E152">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
@@ -3155,13 +3155,13 @@
         <v>132</v>
       </c>
       <c r="B153" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C153">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E153">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
@@ -3169,13 +3169,13 @@
         <v>132</v>
       </c>
       <c r="B154" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C154">
         <v>41</v>
       </c>
       <c r="E154">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
@@ -3183,13 +3183,13 @@
         <v>132</v>
       </c>
       <c r="B155" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C155">
         <v>41</v>
       </c>
       <c r="E155">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
@@ -3197,13 +3197,13 @@
         <v>132</v>
       </c>
       <c r="B156" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C156">
         <v>41</v>
       </c>
       <c r="E156">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
@@ -3211,13 +3211,13 @@
         <v>132</v>
       </c>
       <c r="B157" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C157">
         <v>41</v>
       </c>
       <c r="E157">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
@@ -3225,41 +3225,41 @@
         <v>132</v>
       </c>
       <c r="B158" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C158">
         <v>41</v>
       </c>
       <c r="E158">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>162</v>
+        <v>132</v>
       </c>
       <c r="B159" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C159">
-        <v>152</v>
+        <v>41</v>
       </c>
       <c r="E159">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C160">
-        <v>13</v>
+        <v>152</v>
       </c>
       <c r="E160">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
@@ -3267,13 +3267,13 @@
         <v>164</v>
       </c>
       <c r="B161" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C161">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="E161">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
@@ -3281,13 +3281,13 @@
         <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C162">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="E162">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
@@ -3295,13 +3295,13 @@
         <v>164</v>
       </c>
       <c r="B163" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C163">
-        <v>81</v>
+        <v>17</v>
       </c>
       <c r="E163">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.25">
@@ -3309,27 +3309,27 @@
         <v>164</v>
       </c>
       <c r="B164" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C164">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="E164">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B165" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C165">
-        <v>23</v>
+        <v>76</v>
       </c>
       <c r="E165">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.25">
@@ -3337,13 +3337,13 @@
         <v>170</v>
       </c>
       <c r="B166" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C166">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E166">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.25">
@@ -3351,13 +3351,13 @@
         <v>170</v>
       </c>
       <c r="B167" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C167">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="E167">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.25">
@@ -3365,13 +3365,13 @@
         <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C168">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="E168">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
@@ -3379,27 +3379,27 @@
         <v>170</v>
       </c>
       <c r="B169" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C169">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="E169">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B170" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C170">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="E170">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
@@ -3407,13 +3407,13 @@
         <v>176</v>
       </c>
       <c r="B171" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C171">
-        <v>529</v>
+        <v>54</v>
       </c>
       <c r="E171">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
@@ -3421,13 +3421,13 @@
         <v>176</v>
       </c>
       <c r="B172" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C172">
-        <v>41</v>
+        <v>529</v>
       </c>
       <c r="E172">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
@@ -3435,31 +3435,31 @@
         <v>176</v>
       </c>
       <c r="B173" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C173">
         <v>41</v>
       </c>
       <c r="E173">
-        <v>67</v>
-      </c>
-      <c r="F173" s="1">
-        <f>SUM(C107:C173)</f>
-        <v>3172</v>
+        <v>66</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C174">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="E174">
-        <v>1</v>
+        <v>67</v>
+      </c>
+      <c r="F174" s="1">
+        <f>SUM(C108:C174)</f>
+        <v>3172</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.25">
@@ -3467,13 +3467,13 @@
         <v>181</v>
       </c>
       <c r="B175" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C175">
-        <v>276</v>
+        <v>51</v>
       </c>
       <c r="E175">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.25">
@@ -3481,13 +3481,13 @@
         <v>181</v>
       </c>
       <c r="B176" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C176">
-        <v>61</v>
+        <v>276</v>
       </c>
       <c r="E176">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
@@ -3495,13 +3495,13 @@
         <v>181</v>
       </c>
       <c r="B177" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C177">
-        <v>201</v>
+        <v>61</v>
       </c>
       <c r="E177">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
@@ -3509,13 +3509,13 @@
         <v>181</v>
       </c>
       <c r="B178" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C178">
-        <v>510</v>
+        <v>201</v>
       </c>
       <c r="E178">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
@@ -3523,13 +3523,13 @@
         <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C179">
-        <v>248</v>
+        <v>510</v>
       </c>
       <c r="E179">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
@@ -3537,13 +3537,13 @@
         <v>181</v>
       </c>
       <c r="B180" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C180">
-        <v>622</v>
+        <v>248</v>
       </c>
       <c r="E180">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
@@ -3551,13 +3551,13 @@
         <v>181</v>
       </c>
       <c r="B181" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C181">
-        <v>523</v>
+        <v>622</v>
       </c>
       <c r="E181">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
@@ -3565,13 +3565,13 @@
         <v>181</v>
       </c>
       <c r="B182" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C182">
-        <v>327</v>
+        <v>523</v>
       </c>
       <c r="E182">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
@@ -3579,13 +3579,13 @@
         <v>181</v>
       </c>
       <c r="B183" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C183">
-        <v>178</v>
+        <v>327</v>
       </c>
       <c r="E183">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
@@ -3593,13 +3593,13 @@
         <v>181</v>
       </c>
       <c r="B184" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C184">
-        <v>237</v>
+        <v>178</v>
       </c>
       <c r="E184">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
@@ -3607,13 +3607,13 @@
         <v>181</v>
       </c>
       <c r="B185" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C185">
-        <v>219</v>
+        <v>237</v>
       </c>
       <c r="E185">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.25">
@@ -3621,13 +3621,13 @@
         <v>181</v>
       </c>
       <c r="B186" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C186">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="E186">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
@@ -3635,13 +3635,13 @@
         <v>181</v>
       </c>
       <c r="B187" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C187">
-        <v>219</v>
+        <v>198</v>
       </c>
       <c r="E187">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.25">
@@ -3649,13 +3649,13 @@
         <v>181</v>
       </c>
       <c r="B188" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C188">
-        <v>440</v>
+        <v>219</v>
       </c>
       <c r="E188">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.25">
@@ -3663,13 +3663,13 @@
         <v>181</v>
       </c>
       <c r="B189" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C189">
-        <v>426</v>
+        <v>440</v>
       </c>
       <c r="E189">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
@@ -3677,13 +3677,13 @@
         <v>181</v>
       </c>
       <c r="B190" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C190">
-        <v>292</v>
+        <v>426</v>
       </c>
       <c r="E190">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.25">
@@ -3691,13 +3691,13 @@
         <v>181</v>
       </c>
       <c r="B191" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C191">
-        <v>440</v>
+        <v>292</v>
       </c>
       <c r="E191">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
@@ -3705,249 +3705,263 @@
         <v>181</v>
       </c>
       <c r="B192" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C192">
-        <v>426</v>
+        <v>440</v>
       </c>
       <c r="E192">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>181</v>
       </c>
       <c r="B193" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C193">
-        <v>407</v>
+        <v>426</v>
       </c>
       <c r="E193">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>181</v>
       </c>
       <c r="B194" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C194">
-        <v>423</v>
+        <v>407</v>
       </c>
       <c r="E194">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>181</v>
       </c>
       <c r="B195" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C195">
-        <v>292</v>
+        <v>423</v>
       </c>
       <c r="E195">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>181</v>
       </c>
       <c r="B196" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C196">
-        <v>26</v>
+        <v>292</v>
       </c>
       <c r="E196">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>181</v>
       </c>
       <c r="B197" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C197">
-        <v>452</v>
+        <v>26</v>
       </c>
       <c r="E197">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>181</v>
       </c>
       <c r="B198" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C198">
-        <v>163</v>
+        <v>452</v>
       </c>
       <c r="E198">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>181</v>
       </c>
       <c r="B199" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C199">
-        <v>219</v>
+        <v>163</v>
       </c>
       <c r="E199">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>181</v>
       </c>
       <c r="B200" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C200">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E200">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>181</v>
       </c>
       <c r="B201" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C201">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="E201">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>181</v>
       </c>
       <c r="B202" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C202">
-        <v>238</v>
+        <v>198</v>
       </c>
       <c r="E202">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>181</v>
       </c>
       <c r="B203" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C203">
-        <v>198</v>
+        <v>238</v>
       </c>
       <c r="E203">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>181</v>
       </c>
       <c r="B204" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C204">
-        <v>226</v>
+        <v>198</v>
       </c>
       <c r="E204">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>181</v>
       </c>
       <c r="B205" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C205">
-        <v>267</v>
+        <v>226</v>
       </c>
       <c r="E205">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>181</v>
       </c>
       <c r="B206" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C206">
-        <v>208</v>
+        <v>267</v>
       </c>
       <c r="E206">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>181</v>
       </c>
       <c r="B207" t="s">
+        <v>214</v>
+      </c>
+      <c r="C207">
+        <v>208</v>
+      </c>
+      <c r="E207">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>181</v>
+      </c>
+      <c r="B208" t="s">
         <v>215</v>
       </c>
-      <c r="C207">
+      <c r="C208">
         <v>204</v>
       </c>
-      <c r="E207">
+      <c r="E208">
         <v>34</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A208" t="s">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
         <v>216</v>
       </c>
-      <c r="B208" t="s">
+      <c r="B209" t="s">
         <v>217</v>
       </c>
-      <c r="C208">
+      <c r="C209">
         <v>11</v>
       </c>
-      <c r="E208">
+      <c r="E209">
         <v>35</v>
       </c>
-      <c r="F208" s="1">
-        <f>SUM(C174:C208)</f>
+      <c r="F209" s="1">
+        <f>SUM(C175:C209)</f>
         <v>9639</v>
       </c>
     </row>
-    <row r="209" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B209" t="s">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B210" t="s">
         <v>218</v>
       </c>
-      <c r="F209" s="1">
-        <f>SUM(F1:F208)</f>
+      <c r="F210" s="1">
+        <f>SUM(F2:F209)</f>
         <v>16632</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2025-12-18 Versione  con database ok  per android- aperture db ristrutturate- sviluppato l'inserimento nuovi db di catalogo
</commit_message>
<xml_diff>
--- a/Assets/ElencoVolumiInVecchioDB.xlsx
+++ b/Assets/ElencoVolumiInVecchioDB.xlsx
@@ -13,8 +13,10 @@
   </bookViews>
   <sheets>
     <sheet name="Elenco" sheetId="1" r:id="rId1"/>
+    <sheet name="Cartelle" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="252">
   <si>
     <t>Aebersold</t>
   </si>
@@ -687,6 +689,99 @@
   </si>
   <si>
     <t>NumBrani</t>
+  </si>
+  <si>
+    <t>Cartella</t>
+  </si>
+  <si>
+    <t>sottocartella</t>
+  </si>
+  <si>
+    <t>sottocartella2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimensione </t>
+  </si>
+  <si>
+    <t>S/N</t>
+  </si>
+  <si>
+    <t>Aeber</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Anthol-JAZZ</t>
+  </si>
+  <si>
+    <t>BBAVol1</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>BBAVol2</t>
+  </si>
+  <si>
+    <t>BBAVol3</t>
+  </si>
+  <si>
+    <t>BBAVol4</t>
+  </si>
+  <si>
+    <t>BBAVol5</t>
+  </si>
+  <si>
+    <t>PDF REAL BOOK</t>
+  </si>
+  <si>
+    <t>BookBb</t>
+  </si>
+  <si>
+    <t>BookC</t>
+  </si>
+  <si>
+    <t>BookEb</t>
+  </si>
+  <si>
+    <t>Pigneto</t>
+  </si>
+  <si>
+    <t>SaxQ</t>
+  </si>
+  <si>
+    <t>ProgInterno</t>
+  </si>
+  <si>
+    <t>NumPag</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>potrebbero mancare dei brani verificare</t>
+  </si>
+  <si>
+    <t>ne trova solo 426</t>
+  </si>
+  <si>
+    <t>NON OK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High hope </t>
+  </si>
+  <si>
+    <t>st.thomas 253</t>
+  </si>
+  <si>
+    <t>SCRITTO MALE</t>
+  </si>
+  <si>
+    <t>DOPO 200 c'è un salto</t>
+  </si>
+  <si>
+    <t>ha anche autore</t>
   </si>
 </sst>
 </file>
@@ -1016,22 +1111,29 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F210"/>
+  <dimension ref="A1:L210"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.42578125" customWidth="1"/>
-    <col min="2" max="2" width="80.7109375" customWidth="1"/>
+    <col min="2" max="2" width="56.85546875" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>219</v>
       </c>
       <c r="C1" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>241</v>
+      </c>
+      <c r="F1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1041,11 +1143,11 @@
       <c r="C2">
         <v>12</v>
       </c>
-      <c r="E2">
+      <c r="D2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1055,11 +1157,11 @@
       <c r="C3">
         <v>37</v>
       </c>
-      <c r="E3">
+      <c r="D3">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -1069,11 +1171,11 @@
       <c r="C4">
         <v>37</v>
       </c>
-      <c r="E4">
+      <c r="D4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1083,11 +1185,11 @@
       <c r="C5">
         <v>89</v>
       </c>
-      <c r="E5">
+      <c r="D5">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1097,11 +1199,11 @@
       <c r="C6">
         <v>13</v>
       </c>
-      <c r="E6">
+      <c r="D6">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1111,11 +1213,11 @@
       <c r="C7">
         <v>22</v>
       </c>
-      <c r="E7">
+      <c r="D7">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1125,11 +1227,11 @@
       <c r="C8">
         <v>7</v>
       </c>
-      <c r="E8">
+      <c r="D8">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1139,11 +1241,11 @@
       <c r="C9">
         <v>14</v>
       </c>
-      <c r="E9">
+      <c r="D9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -1153,11 +1255,11 @@
       <c r="C10">
         <v>53</v>
       </c>
-      <c r="E10">
+      <c r="D10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1167,11 +1269,11 @@
       <c r="C11">
         <v>23</v>
       </c>
-      <c r="E11">
+      <c r="D11">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1181,11 +1283,11 @@
       <c r="C12">
         <v>13</v>
       </c>
-      <c r="E12">
+      <c r="D12">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1195,11 +1297,11 @@
       <c r="C13">
         <v>13</v>
       </c>
-      <c r="E13">
+      <c r="D13">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1209,11 +1311,11 @@
       <c r="C14">
         <v>37</v>
       </c>
-      <c r="E14">
+      <c r="D14">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -1223,11 +1325,11 @@
       <c r="C15">
         <v>14</v>
       </c>
-      <c r="E15">
+      <c r="D15">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1237,11 +1339,11 @@
       <c r="C16">
         <v>13</v>
       </c>
-      <c r="E16">
+      <c r="D16">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1251,11 +1353,11 @@
       <c r="C17">
         <v>14</v>
       </c>
-      <c r="E17">
+      <c r="D17">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1265,11 +1367,11 @@
       <c r="C18">
         <v>12</v>
       </c>
-      <c r="E18">
+      <c r="D18">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1279,11 +1381,11 @@
       <c r="C19">
         <v>26</v>
       </c>
-      <c r="E19">
+      <c r="D19">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>0</v>
       </c>
@@ -1293,11 +1395,11 @@
       <c r="C20">
         <v>13</v>
       </c>
-      <c r="E20">
+      <c r="D20">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1307,11 +1409,11 @@
       <c r="C21">
         <v>16</v>
       </c>
-      <c r="E21">
+      <c r="D21">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -1321,11 +1423,11 @@
       <c r="C22">
         <v>29</v>
       </c>
-      <c r="E22">
+      <c r="D22">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1335,11 +1437,11 @@
       <c r="C23">
         <v>21</v>
       </c>
-      <c r="E23">
+      <c r="D23">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1349,11 +1451,11 @@
       <c r="C24">
         <v>4</v>
       </c>
-      <c r="E24">
+      <c r="D24">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1363,11 +1465,11 @@
       <c r="C25">
         <v>12</v>
       </c>
-      <c r="E25">
+      <c r="D25">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -1377,11 +1479,11 @@
       <c r="C26">
         <v>13</v>
       </c>
-      <c r="E26">
+      <c r="D26">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -1391,11 +1493,11 @@
       <c r="C27">
         <v>14</v>
       </c>
-      <c r="E27">
+      <c r="D27">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>0</v>
       </c>
@@ -1405,11 +1507,11 @@
       <c r="C28">
         <v>29</v>
       </c>
-      <c r="E28">
+      <c r="D28">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -1419,11 +1521,11 @@
       <c r="C29">
         <v>13</v>
       </c>
-      <c r="E29">
+      <c r="D29">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>0</v>
       </c>
@@ -1433,11 +1535,11 @@
       <c r="C30">
         <v>11</v>
       </c>
-      <c r="E30">
+      <c r="D30">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>0</v>
       </c>
@@ -1447,11 +1549,11 @@
       <c r="C31">
         <v>15</v>
       </c>
-      <c r="E31">
+      <c r="D31">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>0</v>
       </c>
@@ -1461,11 +1563,11 @@
       <c r="C32">
         <v>49</v>
       </c>
-      <c r="E32">
+      <c r="D32">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
@@ -1475,11 +1577,11 @@
       <c r="C33">
         <v>13</v>
       </c>
-      <c r="E33">
+      <c r="D33">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>0</v>
       </c>
@@ -1489,11 +1591,11 @@
       <c r="C34">
         <v>11</v>
       </c>
-      <c r="E34">
+      <c r="D34">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>0</v>
       </c>
@@ -1503,11 +1605,11 @@
       <c r="C35">
         <v>11</v>
       </c>
-      <c r="E35">
+      <c r="D35">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>0</v>
       </c>
@@ -1517,11 +1619,11 @@
       <c r="C36">
         <v>13</v>
       </c>
-      <c r="E36">
+      <c r="D36">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>0</v>
       </c>
@@ -1531,11 +1633,11 @@
       <c r="C37">
         <v>13</v>
       </c>
-      <c r="E37">
+      <c r="D37">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>0</v>
       </c>
@@ -1545,11 +1647,11 @@
       <c r="C38">
         <v>49</v>
       </c>
-      <c r="E38">
+      <c r="D38">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>0</v>
       </c>
@@ -1559,11 +1661,11 @@
       <c r="C39">
         <v>13</v>
       </c>
-      <c r="E39">
+      <c r="D39">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>0</v>
       </c>
@@ -1573,11 +1675,11 @@
       <c r="C40">
         <v>15</v>
       </c>
-      <c r="E40">
+      <c r="D40">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>0</v>
       </c>
@@ -1587,11 +1689,11 @@
       <c r="C41">
         <v>11</v>
       </c>
-      <c r="E41">
+      <c r="D41">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>0</v>
       </c>
@@ -1601,11 +1703,11 @@
       <c r="C42">
         <v>14</v>
       </c>
-      <c r="E42">
+      <c r="D42">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>0</v>
       </c>
@@ -1615,11 +1717,11 @@
       <c r="C43">
         <v>13</v>
       </c>
-      <c r="E43">
+      <c r="D43">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>0</v>
       </c>
@@ -1629,11 +1731,11 @@
       <c r="C44">
         <v>15</v>
       </c>
-      <c r="E44">
+      <c r="D44">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>0</v>
       </c>
@@ -1643,11 +1745,11 @@
       <c r="C45">
         <v>46</v>
       </c>
-      <c r="E45">
+      <c r="D45">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>0</v>
       </c>
@@ -1657,11 +1759,11 @@
       <c r="C46">
         <v>13</v>
       </c>
-      <c r="E46">
+      <c r="D46">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>0</v>
       </c>
@@ -1671,11 +1773,11 @@
       <c r="C47">
         <v>13</v>
       </c>
-      <c r="E47">
+      <c r="D47">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -1685,11 +1787,11 @@
       <c r="C48">
         <v>11</v>
       </c>
-      <c r="E48">
+      <c r="D48">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>0</v>
       </c>
@@ -1699,11 +1801,11 @@
       <c r="C49">
         <v>34</v>
       </c>
-      <c r="E49">
+      <c r="D49">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>0</v>
       </c>
@@ -1713,11 +1815,11 @@
       <c r="C50">
         <v>4</v>
       </c>
-      <c r="E50">
+      <c r="D50">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>0</v>
       </c>
@@ -1727,11 +1829,11 @@
       <c r="C51">
         <v>10</v>
       </c>
-      <c r="E51">
+      <c r="D51">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>0</v>
       </c>
@@ -1741,11 +1843,11 @@
       <c r="C52">
         <v>29</v>
       </c>
-      <c r="E52">
+      <c r="D52">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>0</v>
       </c>
@@ -1755,11 +1857,11 @@
       <c r="C53">
         <v>25</v>
       </c>
-      <c r="E53">
+      <c r="D53">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>0</v>
       </c>
@@ -1769,11 +1871,11 @@
       <c r="C54">
         <v>21</v>
       </c>
-      <c r="E54">
+      <c r="D54">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>0</v>
       </c>
@@ -1783,11 +1885,11 @@
       <c r="C55">
         <v>8</v>
       </c>
-      <c r="E55">
+      <c r="D55">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>0</v>
       </c>
@@ -1797,11 +1899,11 @@
       <c r="C56">
         <v>9</v>
       </c>
-      <c r="E56">
+      <c r="D56">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>0</v>
       </c>
@@ -1811,11 +1913,11 @@
       <c r="C57">
         <v>25</v>
       </c>
-      <c r="E57">
+      <c r="D57">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>0</v>
       </c>
@@ -1825,11 +1927,11 @@
       <c r="C58">
         <v>28</v>
       </c>
-      <c r="E58">
+      <c r="D58">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>0</v>
       </c>
@@ -1839,11 +1941,11 @@
       <c r="C59">
         <v>17</v>
       </c>
-      <c r="E59">
+      <c r="D59">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>0</v>
       </c>
@@ -1853,11 +1955,11 @@
       <c r="C60">
         <v>9</v>
       </c>
-      <c r="E60">
+      <c r="D60">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>0</v>
       </c>
@@ -1867,11 +1969,11 @@
       <c r="C61">
         <v>13</v>
       </c>
-      <c r="E61">
+      <c r="D61">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>0</v>
       </c>
@@ -1881,11 +1983,11 @@
       <c r="C62">
         <v>6</v>
       </c>
-      <c r="E62">
+      <c r="D62">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>0</v>
       </c>
@@ -1895,11 +1997,11 @@
       <c r="C63">
         <v>17</v>
       </c>
-      <c r="E63">
+      <c r="D63">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>0</v>
       </c>
@@ -1909,11 +2011,11 @@
       <c r="C64">
         <v>18</v>
       </c>
-      <c r="E64">
+      <c r="D64">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>0</v>
       </c>
@@ -1923,11 +2025,11 @@
       <c r="C65">
         <v>9</v>
       </c>
-      <c r="E65">
+      <c r="D65">
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>0</v>
       </c>
@@ -1937,11 +2039,11 @@
       <c r="C66">
         <v>31</v>
       </c>
-      <c r="E66">
+      <c r="D66">
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>0</v>
       </c>
@@ -1951,11 +2053,11 @@
       <c r="C67">
         <v>3</v>
       </c>
-      <c r="E67">
+      <c r="D67">
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>0</v>
       </c>
@@ -1965,11 +2067,11 @@
       <c r="C68">
         <v>15</v>
       </c>
-      <c r="E68">
+      <c r="D68">
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>0</v>
       </c>
@@ -1979,11 +2081,11 @@
       <c r="C69">
         <v>13</v>
       </c>
-      <c r="E69">
+      <c r="D69">
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>0</v>
       </c>
@@ -1993,11 +2095,11 @@
       <c r="C70">
         <v>1</v>
       </c>
-      <c r="E70">
+      <c r="D70">
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>0</v>
       </c>
@@ -2007,11 +2109,11 @@
       <c r="C71">
         <v>18</v>
       </c>
-      <c r="E71">
+      <c r="D71">
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>0</v>
       </c>
@@ -2021,11 +2123,11 @@
       <c r="C72">
         <v>1</v>
       </c>
-      <c r="E72">
+      <c r="D72">
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>0</v>
       </c>
@@ -2035,11 +2137,11 @@
       <c r="C73">
         <v>25</v>
       </c>
-      <c r="E73">
+      <c r="D73">
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>0</v>
       </c>
@@ -2049,11 +2151,11 @@
       <c r="C74">
         <v>19</v>
       </c>
-      <c r="E74">
+      <c r="D74">
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>0</v>
       </c>
@@ -2063,11 +2165,11 @@
       <c r="C75">
         <v>11</v>
       </c>
-      <c r="E75">
+      <c r="D75">
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>0</v>
       </c>
@@ -2077,11 +2179,11 @@
       <c r="C76">
         <v>9</v>
       </c>
-      <c r="E76">
+      <c r="D76">
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>0</v>
       </c>
@@ -2091,11 +2193,11 @@
       <c r="C77">
         <v>31</v>
       </c>
-      <c r="E77">
+      <c r="D77">
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>0</v>
       </c>
@@ -2105,11 +2207,11 @@
       <c r="C78">
         <v>25</v>
       </c>
-      <c r="E78">
+      <c r="D78">
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>0</v>
       </c>
@@ -2119,11 +2221,11 @@
       <c r="C79">
         <v>55</v>
       </c>
-      <c r="E79">
+      <c r="D79">
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>0</v>
       </c>
@@ -2133,11 +2235,11 @@
       <c r="C80">
         <v>55</v>
       </c>
-      <c r="E80">
+      <c r="D80">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>0</v>
       </c>
@@ -2147,11 +2249,11 @@
       <c r="C81">
         <v>10</v>
       </c>
-      <c r="E81">
+      <c r="D81">
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>0</v>
       </c>
@@ -2161,11 +2263,11 @@
       <c r="C82">
         <v>10</v>
       </c>
-      <c r="E82">
+      <c r="D82">
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>0</v>
       </c>
@@ -2175,11 +2277,11 @@
       <c r="C83">
         <v>10</v>
       </c>
-      <c r="E83">
+      <c r="D83">
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>0</v>
       </c>
@@ -2189,11 +2291,11 @@
       <c r="C84">
         <v>36</v>
       </c>
-      <c r="E84">
+      <c r="D84">
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>0</v>
       </c>
@@ -2203,11 +2305,11 @@
       <c r="C85">
         <v>9</v>
       </c>
-      <c r="E85">
+      <c r="D85">
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>0</v>
       </c>
@@ -2217,11 +2319,11 @@
       <c r="C86">
         <v>31</v>
       </c>
-      <c r="E86">
+      <c r="D86">
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>0</v>
       </c>
@@ -2231,11 +2333,14 @@
       <c r="C87">
         <v>18</v>
       </c>
-      <c r="E87">
+      <c r="D87">
         <v>86</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F87" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>0</v>
       </c>
@@ -2245,11 +2350,11 @@
       <c r="C88">
         <v>37</v>
       </c>
-      <c r="E88">
+      <c r="D88">
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>0</v>
       </c>
@@ -2259,11 +2364,11 @@
       <c r="C89">
         <v>17</v>
       </c>
-      <c r="E89">
+      <c r="D89">
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>0</v>
       </c>
@@ -2273,11 +2378,11 @@
       <c r="C90">
         <v>28</v>
       </c>
-      <c r="E90">
+      <c r="D90">
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>0</v>
       </c>
@@ -2287,11 +2392,11 @@
       <c r="C91">
         <v>10</v>
       </c>
-      <c r="E91">
+      <c r="D91">
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>0</v>
       </c>
@@ -2301,11 +2406,11 @@
       <c r="C92">
         <v>10</v>
       </c>
-      <c r="E92">
+      <c r="D92">
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>0</v>
       </c>
@@ -2315,11 +2420,11 @@
       <c r="C93">
         <v>15</v>
       </c>
-      <c r="E93">
+      <c r="D93">
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>0</v>
       </c>
@@ -2329,11 +2434,11 @@
       <c r="C94">
         <v>10</v>
       </c>
-      <c r="E94">
+      <c r="D94">
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>0</v>
       </c>
@@ -2343,11 +2448,11 @@
       <c r="C95">
         <v>37</v>
       </c>
-      <c r="E95">
+      <c r="D95">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>0</v>
       </c>
@@ -2357,7 +2462,7 @@
       <c r="C96">
         <v>35</v>
       </c>
-      <c r="E96">
+      <c r="D96">
         <v>95</v>
       </c>
     </row>
@@ -2371,7 +2476,7 @@
       <c r="C97">
         <v>27</v>
       </c>
-      <c r="E97">
+      <c r="D97">
         <v>96</v>
       </c>
     </row>
@@ -2385,7 +2490,7 @@
       <c r="C98">
         <v>13</v>
       </c>
-      <c r="E98">
+      <c r="D98">
         <v>97</v>
       </c>
     </row>
@@ -2399,7 +2504,7 @@
       <c r="C99">
         <v>13</v>
       </c>
-      <c r="E99">
+      <c r="D99">
         <v>98</v>
       </c>
     </row>
@@ -2413,7 +2518,7 @@
       <c r="C100">
         <v>28</v>
       </c>
-      <c r="E100">
+      <c r="D100">
         <v>99</v>
       </c>
     </row>
@@ -2427,7 +2532,7 @@
       <c r="C101">
         <v>23</v>
       </c>
-      <c r="E101">
+      <c r="D101">
         <v>100</v>
       </c>
     </row>
@@ -2441,7 +2546,7 @@
       <c r="C102">
         <v>40</v>
       </c>
-      <c r="E102">
+      <c r="D102">
         <v>101</v>
       </c>
     </row>
@@ -2455,7 +2560,7 @@
       <c r="C103">
         <v>40</v>
       </c>
-      <c r="E103">
+      <c r="D103">
         <v>102</v>
       </c>
     </row>
@@ -2469,7 +2574,7 @@
       <c r="C104">
         <v>39</v>
       </c>
-      <c r="E104">
+      <c r="D104">
         <v>103</v>
       </c>
     </row>
@@ -2483,7 +2588,7 @@
       <c r="C105">
         <v>23</v>
       </c>
-      <c r="E105">
+      <c r="D105">
         <v>104</v>
       </c>
     </row>
@@ -2497,10 +2602,10 @@
       <c r="C106">
         <v>9</v>
       </c>
-      <c r="E106">
+      <c r="D106">
         <v>105</v>
       </c>
-      <c r="F106" s="1">
+      <c r="E106" s="1">
         <f>SUM(C2:C106)</f>
         <v>2134</v>
       </c>
@@ -2515,9 +2620,12 @@
       <c r="C107">
         <v>1687</v>
       </c>
-      <c r="F107" s="1">
+      <c r="E107" s="1">
         <f>SUM(C107)</f>
         <v>1687</v>
+      </c>
+      <c r="F107" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -2530,8 +2638,11 @@
       <c r="C108">
         <v>201</v>
       </c>
-      <c r="E108">
+      <c r="D108">
         <v>1</v>
+      </c>
+      <c r="F108" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -2544,7 +2655,7 @@
       <c r="C109">
         <v>13</v>
       </c>
-      <c r="E109">
+      <c r="D109">
         <v>2</v>
       </c>
     </row>
@@ -2558,7 +2669,7 @@
       <c r="C110">
         <v>18</v>
       </c>
-      <c r="E110">
+      <c r="D110">
         <v>3</v>
       </c>
     </row>
@@ -2572,7 +2683,7 @@
       <c r="C111">
         <v>16</v>
       </c>
-      <c r="E111">
+      <c r="D111">
         <v>4</v>
       </c>
     </row>
@@ -2586,11 +2697,11 @@
       <c r="C112">
         <v>21</v>
       </c>
-      <c r="E112">
+      <c r="D112">
         <v>5</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>108</v>
       </c>
@@ -2600,11 +2711,11 @@
       <c r="C113">
         <v>23</v>
       </c>
-      <c r="E113">
+      <c r="D113">
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>108</v>
       </c>
@@ -2614,11 +2725,11 @@
       <c r="C114">
         <v>12</v>
       </c>
-      <c r="E114">
+      <c r="D114">
         <v>7</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>108</v>
       </c>
@@ -2628,11 +2739,11 @@
       <c r="C115">
         <v>12</v>
       </c>
-      <c r="E115">
+      <c r="D115">
         <v>8</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>108</v>
       </c>
@@ -2642,11 +2753,11 @@
       <c r="C116">
         <v>12</v>
       </c>
-      <c r="E116">
+      <c r="D116">
         <v>9</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>108</v>
       </c>
@@ -2656,11 +2767,11 @@
       <c r="C117">
         <v>49</v>
       </c>
-      <c r="E117">
+      <c r="D117">
         <v>10</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>108</v>
       </c>
@@ -2670,11 +2781,11 @@
       <c r="C118">
         <v>75</v>
       </c>
-      <c r="E118">
+      <c r="D118">
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>108</v>
       </c>
@@ -2684,11 +2795,11 @@
       <c r="C119">
         <v>20</v>
       </c>
-      <c r="E119">
+      <c r="D119">
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>108</v>
       </c>
@@ -2698,11 +2809,11 @@
       <c r="C120">
         <v>21</v>
       </c>
-      <c r="E120">
+      <c r="D120">
         <v>13</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>108</v>
       </c>
@@ -2712,11 +2823,11 @@
       <c r="C121">
         <v>41</v>
       </c>
-      <c r="E121">
+      <c r="D121">
         <v>14</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>108</v>
       </c>
@@ -2726,11 +2837,11 @@
       <c r="C122">
         <v>37</v>
       </c>
-      <c r="E122">
+      <c r="D122">
         <v>15</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>108</v>
       </c>
@@ -2740,11 +2851,11 @@
       <c r="C123">
         <v>41</v>
       </c>
-      <c r="E123">
+      <c r="D123">
         <v>16</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>108</v>
       </c>
@@ -2754,11 +2865,11 @@
       <c r="C124">
         <v>11</v>
       </c>
-      <c r="E124">
+      <c r="D124">
         <v>17</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>108</v>
       </c>
@@ -2768,11 +2879,11 @@
       <c r="C125">
         <v>13</v>
       </c>
-      <c r="E125">
+      <c r="D125">
         <v>18</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>108</v>
       </c>
@@ -2782,11 +2893,11 @@
       <c r="C126">
         <v>37</v>
       </c>
-      <c r="E126">
+      <c r="D126">
         <v>19</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>108</v>
       </c>
@@ -2796,11 +2907,11 @@
       <c r="C127">
         <v>41</v>
       </c>
-      <c r="E127">
+      <c r="D127">
         <v>20</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>108</v>
       </c>
@@ -2810,11 +2921,11 @@
       <c r="C128">
         <v>9</v>
       </c>
-      <c r="E128">
+      <c r="D128">
         <v>21</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>108</v>
       </c>
@@ -2824,11 +2935,11 @@
       <c r="C129">
         <v>15</v>
       </c>
-      <c r="E129">
+      <c r="D129">
         <v>22</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>108</v>
       </c>
@@ -2838,11 +2949,11 @@
       <c r="C130">
         <v>107</v>
       </c>
-      <c r="E130">
+      <c r="D130">
         <v>23</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>132</v>
       </c>
@@ -2852,11 +2963,11 @@
       <c r="C131">
         <v>41</v>
       </c>
-      <c r="E131">
+      <c r="D131">
         <v>24</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>132</v>
       </c>
@@ -2866,11 +2977,11 @@
       <c r="C132">
         <v>41</v>
       </c>
-      <c r="E132">
+      <c r="D132">
         <v>25</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>132</v>
       </c>
@@ -2880,11 +2991,11 @@
       <c r="C133">
         <v>41</v>
       </c>
-      <c r="E133">
+      <c r="D133">
         <v>26</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>132</v>
       </c>
@@ -2894,11 +3005,11 @@
       <c r="C134">
         <v>41</v>
       </c>
-      <c r="E134">
+      <c r="D134">
         <v>27</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>132</v>
       </c>
@@ -2908,11 +3019,11 @@
       <c r="C135">
         <v>41</v>
       </c>
-      <c r="E135">
+      <c r="D135">
         <v>28</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>132</v>
       </c>
@@ -2922,11 +3033,11 @@
       <c r="C136">
         <v>21</v>
       </c>
-      <c r="E136">
+      <c r="D136">
         <v>29</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>132</v>
       </c>
@@ -2936,11 +3047,11 @@
       <c r="C137">
         <v>41</v>
       </c>
-      <c r="E137">
+      <c r="D137">
         <v>30</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>132</v>
       </c>
@@ -2950,11 +3061,11 @@
       <c r="C138">
         <v>41</v>
       </c>
-      <c r="E138">
+      <c r="D138">
         <v>31</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>132</v>
       </c>
@@ -2964,11 +3075,11 @@
       <c r="C139">
         <v>41</v>
       </c>
-      <c r="E139">
+      <c r="D139">
         <v>32</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>132</v>
       </c>
@@ -2978,11 +3089,11 @@
       <c r="C140">
         <v>41</v>
       </c>
-      <c r="E140">
+      <c r="D140">
         <v>33</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>132</v>
       </c>
@@ -2992,11 +3103,11 @@
       <c r="C141">
         <v>41</v>
       </c>
-      <c r="E141">
+      <c r="D141">
         <v>34</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>132</v>
       </c>
@@ -3006,11 +3117,11 @@
       <c r="C142">
         <v>37</v>
       </c>
-      <c r="E142">
+      <c r="D142">
         <v>35</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>132</v>
       </c>
@@ -3020,11 +3131,11 @@
       <c r="C143">
         <v>41</v>
       </c>
-      <c r="E143">
+      <c r="D143">
         <v>36</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>132</v>
       </c>
@@ -3034,11 +3145,11 @@
       <c r="C144">
         <v>41</v>
       </c>
-      <c r="E144">
+      <c r="D144">
         <v>37</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>132</v>
       </c>
@@ -3048,11 +3159,11 @@
       <c r="C145">
         <v>33</v>
       </c>
-      <c r="E145">
+      <c r="D145">
         <v>38</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>132</v>
       </c>
@@ -3062,11 +3173,11 @@
       <c r="C146">
         <v>41</v>
       </c>
-      <c r="E146">
+      <c r="D146">
         <v>39</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>132</v>
       </c>
@@ -3076,11 +3187,11 @@
       <c r="C147">
         <v>41</v>
       </c>
-      <c r="E147">
+      <c r="D147">
         <v>40</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>132</v>
       </c>
@@ -3090,11 +3201,11 @@
       <c r="C148">
         <v>41</v>
       </c>
-      <c r="E148">
+      <c r="D148">
         <v>41</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>132</v>
       </c>
@@ -3104,11 +3215,11 @@
       <c r="C149">
         <v>41</v>
       </c>
-      <c r="E149">
+      <c r="D149">
         <v>42</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>132</v>
       </c>
@@ -3118,11 +3229,11 @@
       <c r="C150">
         <v>41</v>
       </c>
-      <c r="E150">
+      <c r="D150">
         <v>43</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>132</v>
       </c>
@@ -3132,11 +3243,11 @@
       <c r="C151">
         <v>41</v>
       </c>
-      <c r="E151">
+      <c r="D151">
         <v>44</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>132</v>
       </c>
@@ -3146,11 +3257,11 @@
       <c r="C152">
         <v>41</v>
       </c>
-      <c r="E152">
+      <c r="D152">
         <v>45</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>132</v>
       </c>
@@ -3160,11 +3271,11 @@
       <c r="C153">
         <v>37</v>
       </c>
-      <c r="E153">
+      <c r="D153">
         <v>46</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>132</v>
       </c>
@@ -3174,11 +3285,11 @@
       <c r="C154">
         <v>41</v>
       </c>
-      <c r="E154">
+      <c r="D154">
         <v>47</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>132</v>
       </c>
@@ -3188,11 +3299,11 @@
       <c r="C155">
         <v>41</v>
       </c>
-      <c r="E155">
+      <c r="D155">
         <v>48</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>132</v>
       </c>
@@ -3202,11 +3313,11 @@
       <c r="C156">
         <v>41</v>
       </c>
-      <c r="E156">
+      <c r="D156">
         <v>49</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>132</v>
       </c>
@@ -3216,11 +3327,11 @@
       <c r="C157">
         <v>41</v>
       </c>
-      <c r="E157">
+      <c r="D157">
         <v>50</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>132</v>
       </c>
@@ -3230,11 +3341,11 @@
       <c r="C158">
         <v>41</v>
       </c>
-      <c r="E158">
+      <c r="D158">
         <v>51</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>132</v>
       </c>
@@ -3244,11 +3355,11 @@
       <c r="C159">
         <v>41</v>
       </c>
-      <c r="E159">
+      <c r="D159">
         <v>52</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>162</v>
       </c>
@@ -3258,11 +3369,11 @@
       <c r="C160">
         <v>152</v>
       </c>
-      <c r="E160">
+      <c r="D160">
         <v>53</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>164</v>
       </c>
@@ -3272,11 +3383,11 @@
       <c r="C161">
         <v>13</v>
       </c>
-      <c r="E161">
+      <c r="D161">
         <v>54</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>164</v>
       </c>
@@ -3286,11 +3397,11 @@
       <c r="C162">
         <v>59</v>
       </c>
-      <c r="E162">
+      <c r="D162">
         <v>55</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>164</v>
       </c>
@@ -3300,11 +3411,11 @@
       <c r="C163">
         <v>17</v>
       </c>
-      <c r="E163">
+      <c r="D163">
         <v>56</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>164</v>
       </c>
@@ -3314,11 +3425,11 @@
       <c r="C164">
         <v>81</v>
       </c>
-      <c r="E164">
+      <c r="D164">
         <v>57</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>164</v>
       </c>
@@ -3328,11 +3439,11 @@
       <c r="C165">
         <v>76</v>
       </c>
-      <c r="E165">
+      <c r="D165">
         <v>58</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>170</v>
       </c>
@@ -3342,11 +3453,11 @@
       <c r="C166">
         <v>23</v>
       </c>
-      <c r="E166">
+      <c r="D166">
         <v>59</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>170</v>
       </c>
@@ -3356,11 +3467,11 @@
       <c r="C167">
         <v>26</v>
       </c>
-      <c r="E167">
+      <c r="D167">
         <v>60</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>170</v>
       </c>
@@ -3370,11 +3481,11 @@
       <c r="C168">
         <v>15</v>
       </c>
-      <c r="E168">
+      <c r="D168">
         <v>61</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>170</v>
       </c>
@@ -3384,11 +3495,11 @@
       <c r="C169">
         <v>27</v>
       </c>
-      <c r="E169">
+      <c r="D169">
         <v>62</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>170</v>
       </c>
@@ -3398,11 +3509,11 @@
       <c r="C170">
         <v>20</v>
       </c>
-      <c r="E170">
+      <c r="D170">
         <v>63</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>176</v>
       </c>
@@ -3412,11 +3523,11 @@
       <c r="C171">
         <v>54</v>
       </c>
-      <c r="E171">
+      <c r="D171">
         <v>64</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>176</v>
       </c>
@@ -3426,11 +3537,11 @@
       <c r="C172">
         <v>529</v>
       </c>
-      <c r="E172">
+      <c r="D172">
         <v>65</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>176</v>
       </c>
@@ -3440,11 +3551,11 @@
       <c r="C173">
         <v>41</v>
       </c>
-      <c r="E173">
+      <c r="D173">
         <v>66</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>176</v>
       </c>
@@ -3454,15 +3565,15 @@
       <c r="C174">
         <v>41</v>
       </c>
-      <c r="E174">
+      <c r="D174">
         <v>67</v>
       </c>
-      <c r="F174" s="1">
+      <c r="E174" s="1">
         <f>SUM(C108:C174)</f>
         <v>3172</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>181</v>
       </c>
@@ -3472,11 +3583,11 @@
       <c r="C175">
         <v>51</v>
       </c>
-      <c r="E175">
+      <c r="D175">
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>181</v>
       </c>
@@ -3486,11 +3597,11 @@
       <c r="C176">
         <v>276</v>
       </c>
-      <c r="E176">
+      <c r="D176">
         <v>2</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>181</v>
       </c>
@@ -3500,11 +3611,11 @@
       <c r="C177">
         <v>61</v>
       </c>
-      <c r="E177">
+      <c r="D177">
         <v>3</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>181</v>
       </c>
@@ -3514,11 +3625,11 @@
       <c r="C178">
         <v>201</v>
       </c>
-      <c r="E178">
+      <c r="D178">
         <v>4</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>181</v>
       </c>
@@ -3528,11 +3639,11 @@
       <c r="C179">
         <v>510</v>
       </c>
-      <c r="E179">
+      <c r="D179">
         <v>5</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>181</v>
       </c>
@@ -3542,11 +3653,11 @@
       <c r="C180">
         <v>248</v>
       </c>
-      <c r="E180">
+      <c r="D180">
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>181</v>
       </c>
@@ -3556,11 +3667,11 @@
       <c r="C181">
         <v>622</v>
       </c>
-      <c r="E181">
+      <c r="D181">
         <v>7</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>181</v>
       </c>
@@ -3570,11 +3681,11 @@
       <c r="C182">
         <v>523</v>
       </c>
-      <c r="E182">
+      <c r="D182">
         <v>8</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>181</v>
       </c>
@@ -3584,11 +3695,11 @@
       <c r="C183">
         <v>327</v>
       </c>
-      <c r="E183">
+      <c r="D183">
         <v>9</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>181</v>
       </c>
@@ -3598,11 +3709,11 @@
       <c r="C184">
         <v>178</v>
       </c>
-      <c r="E184">
+      <c r="D184">
         <v>10</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>181</v>
       </c>
@@ -3612,11 +3723,14 @@
       <c r="C185">
         <v>237</v>
       </c>
-      <c r="E185">
+      <c r="D185">
         <v>11</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F185" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>181</v>
       </c>
@@ -3626,11 +3740,14 @@
       <c r="C186">
         <v>219</v>
       </c>
-      <c r="E186">
+      <c r="D186">
         <v>12</v>
       </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F186" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>181</v>
       </c>
@@ -3640,11 +3757,14 @@
       <c r="C187">
         <v>198</v>
       </c>
-      <c r="E187">
+      <c r="D187">
         <v>13</v>
       </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F187" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>181</v>
       </c>
@@ -3654,11 +3774,17 @@
       <c r="C188">
         <v>219</v>
       </c>
-      <c r="E188">
+      <c r="D188">
         <v>14</v>
       </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F188" t="s">
+        <v>243</v>
+      </c>
+      <c r="G188" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>181</v>
       </c>
@@ -3668,11 +3794,14 @@
       <c r="C189">
         <v>440</v>
       </c>
-      <c r="E189">
+      <c r="D189">
         <v>15</v>
       </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F189" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>181</v>
       </c>
@@ -3682,11 +3811,17 @@
       <c r="C190">
         <v>426</v>
       </c>
-      <c r="E190">
+      <c r="D190">
         <v>16</v>
       </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F190" t="s">
+        <v>243</v>
+      </c>
+      <c r="G190" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>181</v>
       </c>
@@ -3696,11 +3831,14 @@
       <c r="C191">
         <v>292</v>
       </c>
-      <c r="E191">
+      <c r="D191">
         <v>17</v>
       </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F191" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>181</v>
       </c>
@@ -3710,11 +3848,14 @@
       <c r="C192">
         <v>440</v>
       </c>
-      <c r="E192">
+      <c r="D192">
         <v>18</v>
       </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F192" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>181</v>
       </c>
@@ -3724,11 +3865,14 @@
       <c r="C193">
         <v>426</v>
       </c>
-      <c r="E193">
+      <c r="D193">
         <v>19</v>
       </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F193" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>181</v>
       </c>
@@ -3738,11 +3882,14 @@
       <c r="C194">
         <v>407</v>
       </c>
-      <c r="E194">
+      <c r="D194">
         <v>20</v>
       </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F194" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>181</v>
       </c>
@@ -3752,11 +3899,14 @@
       <c r="C195">
         <v>423</v>
       </c>
-      <c r="E195">
+      <c r="D195">
         <v>21</v>
       </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F195" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>181</v>
       </c>
@@ -3766,11 +3916,29 @@
       <c r="C196">
         <v>292</v>
       </c>
-      <c r="E196">
+      <c r="D196">
         <v>22</v>
       </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F196" t="s">
+        <v>246</v>
+      </c>
+      <c r="G196" t="s">
+        <v>247</v>
+      </c>
+      <c r="H196">
+        <v>108</v>
+      </c>
+      <c r="I196">
+        <v>2</v>
+      </c>
+      <c r="J196" t="s">
+        <v>248</v>
+      </c>
+      <c r="L196">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>181</v>
       </c>
@@ -3780,11 +3948,17 @@
       <c r="C197">
         <v>26</v>
       </c>
-      <c r="E197">
+      <c r="D197">
         <v>23</v>
       </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F197" t="s">
+        <v>243</v>
+      </c>
+      <c r="G197" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>181</v>
       </c>
@@ -3794,11 +3968,20 @@
       <c r="C198">
         <v>452</v>
       </c>
-      <c r="E198">
+      <c r="D198">
         <v>24</v>
       </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F198" t="s">
+        <v>246</v>
+      </c>
+      <c r="G198" t="s">
+        <v>250</v>
+      </c>
+      <c r="I198">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>181</v>
       </c>
@@ -3808,11 +3991,14 @@
       <c r="C199">
         <v>163</v>
       </c>
-      <c r="E199">
+      <c r="D199">
         <v>25</v>
       </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F199" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>181</v>
       </c>
@@ -3822,11 +4008,14 @@
       <c r="C200">
         <v>219</v>
       </c>
-      <c r="E200">
+      <c r="D200">
         <v>26</v>
       </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F200" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>181</v>
       </c>
@@ -3836,11 +4025,14 @@
       <c r="C201">
         <v>213</v>
       </c>
-      <c r="E201">
+      <c r="D201">
         <v>27</v>
       </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F201" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>181</v>
       </c>
@@ -3850,11 +4042,14 @@
       <c r="C202">
         <v>198</v>
       </c>
-      <c r="E202">
+      <c r="D202">
         <v>28</v>
       </c>
-    </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F202" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>181</v>
       </c>
@@ -3864,11 +4059,14 @@
       <c r="C203">
         <v>238</v>
       </c>
-      <c r="E203">
+      <c r="D203">
         <v>29</v>
       </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F203" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>181</v>
       </c>
@@ -3878,11 +4076,14 @@
       <c r="C204">
         <v>198</v>
       </c>
-      <c r="E204">
+      <c r="D204">
         <v>30</v>
       </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F204" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>181</v>
       </c>
@@ -3892,11 +4093,14 @@
       <c r="C205">
         <v>226</v>
       </c>
-      <c r="E205">
+      <c r="D205">
         <v>31</v>
       </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F205" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="206" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>181</v>
       </c>
@@ -3906,11 +4110,14 @@
       <c r="C206">
         <v>267</v>
       </c>
-      <c r="E206">
+      <c r="D206">
         <v>32</v>
       </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F206" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="207" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>181</v>
       </c>
@@ -3920,11 +4127,14 @@
       <c r="C207">
         <v>208</v>
       </c>
-      <c r="E207">
+      <c r="D207">
         <v>33</v>
       </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F207" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>181</v>
       </c>
@@ -3934,11 +4144,17 @@
       <c r="C208">
         <v>204</v>
       </c>
-      <c r="E208">
+      <c r="D208">
         <v>34</v>
       </c>
-    </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F208" t="s">
+        <v>243</v>
+      </c>
+      <c r="G208" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>216</v>
       </c>
@@ -3948,20 +4164,20 @@
       <c r="C209">
         <v>11</v>
       </c>
-      <c r="E209">
+      <c r="D209">
         <v>35</v>
       </c>
-      <c r="F209" s="1">
+      <c r="E209" s="1">
         <f>SUM(C175:C209)</f>
         <v>9639</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B210" t="s">
         <v>218</v>
       </c>
-      <c r="F210" s="1">
-        <f>SUM(F2:F209)</f>
+      <c r="E210" s="1">
+        <f>SUM(E2:E209)</f>
         <v>16632</v>
       </c>
     </row>
@@ -3969,4 +4185,251 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="58" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D1" t="s">
+        <v>224</v>
+      </c>
+      <c r="E1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D2">
+        <v>785</v>
+      </c>
+      <c r="E2" t="s">
+        <v>227</v>
+      </c>
+      <c r="F2">
+        <f>IF(E2="S",D2,0)</f>
+        <v>785</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>228</v>
+      </c>
+      <c r="D3">
+        <v>52.6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>227</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F14" si="0">IF(E3="S",D3,0)</f>
+        <v>52.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D4">
+        <v>306</v>
+      </c>
+      <c r="E4" t="s">
+        <v>230</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>231</v>
+      </c>
+      <c r="D5">
+        <v>319</v>
+      </c>
+      <c r="E5" t="s">
+        <v>230</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>232</v>
+      </c>
+      <c r="D6">
+        <v>405</v>
+      </c>
+      <c r="E6" t="s">
+        <v>230</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7">
+        <v>364</v>
+      </c>
+      <c r="E7" t="s">
+        <v>230</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8">
+        <v>350</v>
+      </c>
+      <c r="E8" t="s">
+        <v>230</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9">
+        <v>1530</v>
+      </c>
+      <c r="E9" t="s">
+        <v>227</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" t="s">
+        <v>236</v>
+      </c>
+      <c r="D10">
+        <v>270</v>
+      </c>
+      <c r="E10" t="s">
+        <v>227</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>270</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>235</v>
+      </c>
+      <c r="B11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D11">
+        <v>721</v>
+      </c>
+      <c r="E11" t="s">
+        <v>227</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>721</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>235</v>
+      </c>
+      <c r="B12" t="s">
+        <v>238</v>
+      </c>
+      <c r="D12">
+        <v>271</v>
+      </c>
+      <c r="E12" t="s">
+        <v>227</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>271</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>239</v>
+      </c>
+      <c r="D13">
+        <v>141</v>
+      </c>
+      <c r="E13" t="s">
+        <v>230</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>240</v>
+      </c>
+      <c r="D14">
+        <v>2020</v>
+      </c>
+      <c r="E14" t="s">
+        <v>230</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <f>SUM(D2:D14)</f>
+        <v>7534.6</v>
+      </c>
+      <c r="F15">
+        <f>SUM(F2:F14)</f>
+        <v>3629.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
2025-12-25 Refactor: Rinominato progetto in 'livescore' e ottimizzazione database
</commit_message>
<xml_diff>
--- a/Assets/ElencoVolumiInVecchioDB.xlsx
+++ b/Assets/ElencoVolumiInVecchioDB.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12960" windowHeight="5790" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12960" windowHeight="5790"/>
   </bookViews>
   <sheets>
     <sheet name="Elenco" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,6 @@
     <sheet name="Monografie PDF" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="464">
   <si>
     <t>Aebersold</t>
   </si>
@@ -1419,6 +1418,9 @@
   </si>
   <si>
     <t>Omnibook!A1</t>
+  </si>
+  <si>
+    <t>non OK</t>
   </si>
 </sst>
 </file>
@@ -3912,6 +3914,9 @@
       <c r="D152">
         <v>45</v>
       </c>
+      <c r="F152" t="s">
+        <v>463</v>
+      </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" t="s">

</xml_diff>